<commit_message>
Add economy simulation report for 2026-09-16
- Introduced a comprehensive report detailing the economy balance simulation for the specified date.
- Included sections on blockers, critical findings, per-check results, summary verdicts, and recommendations.
- Highlighted key metrics such as lifetime gold income, gold sink balance, material income vs spend, and facility cost curves.
- Provided actionable recommendations to address identified issues, including facility costs and overleveled gold penalty scope.
</commit_message>
<xml_diff>
--- a/docs/CTRBLXAI_Development_Roadmap.xlsx
+++ b/docs/CTRBLXAI_Development_Roadmap.xlsx
@@ -16,9 +16,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice 4 - Loadouts Saving" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice 5 - Procedural Maps" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice 6 - Content Expansion" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How To Use" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice 7 - Visual Polish" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice 8 - Guild Base" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice 7 - Visuals UI" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice 8 - Base Multiplayer" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice 9 - Dungeons" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How To Use" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -440,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -685,12 +686,828 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Visuals &amp; UI</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Battle animations, mobile UI, CT timeline bar, polish</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>⬜ Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Base Building &amp; Multiplayer</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>HQ facilities, base progression, multiplayer/co-op, live service</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>⬜ Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Dungeons</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>STS-style branching paths, exclusive loot, avatar mutation events</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>⬜ Not started</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="72" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Goal:</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Polish visual presentation, battle animations, and UI/UX for mobile. Make the game look and feel professional.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Done When:</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Battles look smooth, touch controls feel responsive, CT timeline is readable, and the game looks like a finished product.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Battle animations: attack, skill cast, hit reaction, KO</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>CT timeline bar at top of screen (Mana Khemia style) with unit portraits</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Each action resolves visually immediately before next prompt (no batching)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Targeting by tile tap — click tile selects occupant</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>All UI interactions use tap/touch events only (no hover patterns)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Damage numbers float above units</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Status effect icons visible on affected units</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Skill selection UI polished for mobile (large tap targets)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Map camera controls (pinch zoom, pan, rotate)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Unit info panel (tap unit to see stats, skills, status)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Battle result screen with rewards summary</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Menu/inventory UI polished for mobile</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Sound effects for actions, hits, KO</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Background music per biome</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Loading screen during map pre-generation</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="72" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Goal:</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Build the HQ facility system, base progression, and multiplayer features. Players have a persistent home base that grows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Done When:</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Players can upgrade facilities, access all HQ features, and interact with other players.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>HQ base rendered as a visitable location</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Guild Hall facility (core HQ hub)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Tavern facility (recruitment)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Blacksmith facility (item upgrades, cap +10/level)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Merchant facility (buy/sell)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Quest Board facility (quest selection)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Workshop facility</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Training Ground facility</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Trophy Hall facility (achievements display)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Dungeon facility (unlocks dungeon access — upgradeable)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Facility upgrade system (gold cost, level requirements)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Dungeon facility upgrades: biome selection, difficulty, recovery</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Base progression tied to Guild Level</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Multiplayer/co-op: visit other players' bases</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Multiplayer/co-op: cooperative battles</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Live service features (seasonal events, leaderboards)</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="72" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Goal:</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Build the STS-style dungeon system. Branching node paths, risk/reward, exclusive loot, and avatar mutation events.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Done When:</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Players can enter dungeons, navigate branching paths, encounter varied nodes, find exclusive rewards, and experience avatar perk/drawback mutations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Dungeon node-graph generation (branching paths, not tile grid)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Node types implemented: battle, event, shop, rest, treasure, boss</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Player chooses path at each fork (visual map)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Dungeon map UI (STS-style connected node display)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Battle nodes use existing combat system on generated maps</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Event nodes: random events with choices and consequences</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Shop nodes: spend gold on dungeon-specific items</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Rest nodes: heal/recover between battles</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Treasure nodes: exclusive loot (furniture, rare items)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Boss nodes: harder battle with guaranteed exclusive reward</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Dungeon-exclusive loot tables (separate from quest loot)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Team-wide temporary buffs/debuffs from dungeon events</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Avatar perk/drawback mutation events (rare, swap only)</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Dungeon run state tracking (progress persisted mid-run)</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Dungeon facility upgrade integration (biome, difficulty, recovery)</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Dungeon difficulty scaling per facility level</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Multiple dungeon biomes available based on facility upgrades</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -784,3059 +1601,6 @@
       <c r="B7" t="inlineStr">
         <is>
           <t>Track issues, decisions, or things to revisit.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C186"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Goal:</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>VISUALS, LAYOUT, THEMES, ASSETS, AND PRESENTATION — make the game look and feel good</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Done When:</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>A new player watches 30 seconds of gameplay and it looks like a real game, not a prototype. All visual work consumes authoritative data from other slices.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Task</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Terrain tiles have distinct materials per type (grass, stone, sand, water, etc.)</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Elevation visually reads clearly (cliff faces, ramps, height layers)</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Each biome has a unique visual palette and props</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Map props/objects placed (trees, rocks, buildings, fences)</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Lighting per biome (warm plains, cold highlands, dark caves)</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Unit models distinct per weapon archetype or role</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Attack animations (swing, thrust, cast, shoot)</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Skill VFX (fire burst, heal glow, poison cloud, etc.)</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Status effect visual indicators on units</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>CT timeline bar UI (Mana Khemia style, top of screen)</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>🔄</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>BattleHUD.lua expanded from 37KB to 66KB; UpdateTimeline exists</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Skill Card selection UI polished</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>🔄</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>BattleHUD.ShowSkillList/ShowSkillDetail exist</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Damage/healing numbers styled (floating, color-coded)</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>🔄</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>showDamageText/showFloatingText exist in BattleVisualClient</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Camera system (follow active unit, smooth transitions)</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>🔄 Desktop Verified</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Stage 1 Desktop Checkpoint. Commit: e8dcc977. Mobile pending.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Menu/loadout UI visual design</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>🔄</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>LoadoutScreen.lua (76KB) created; LoadoutController.client.lua exists</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Sound effects (hit, heal, status apply, UI clicks)</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Music per biome or battle phase</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="21"/>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>═══ STAGE 1: TACTICAL CAMERA ═══</t>
-        </is>
-      </c>
-    </row>
-    <row r="23"/>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>--- Desktop Checkpoint (VERIFIED) ---</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Commit: e8dcc9774d494f86d7c44be3fec994fbdef6ec63</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Tactical camera fixed pitch: 50 degrees</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Tactical camera fixed FieldOfView: 55 degrees</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Camera distances: Min 38, Default 53, Max 96 studs</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Playable battle-grid bounds: X -20..20, Z -20..20</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Two-tile camera pan margin</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Screen-relative WASD panning</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Screen-relative arrow-key panning</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Diagonal movement normalization</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Desktop right-drag camera panning</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Q/E rotation in fixed 45-degree steps</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Mouse-wheel zoom</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Left-click tile selection</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>HUD panels block battlefield clicks</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>HUD panels block camera drags</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>Focus Active camera recovery</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>Reset Camera recovery</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>Battle-only tactical camera activation</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>Desktop bootstrap after declaration-order correction</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>Studio-only DEV CAMERA TEST panel</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="44"/>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>--- Mobile Validation (PENDING) ---</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>Studio Emulator two-finger mode issue; not a confirmed code failure</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>Mobile single-tap tile selection</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>Pending reliable single-touch UAT</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>Mobile single-finger camera pan</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>Mobile two-finger fixed-angle rotation</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>Mobile pinch zoom</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>Mobile gesture input blocking</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="51"/>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>--- Deferred to Slice 7 View Mode ---</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>⏳</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>Focus Selected camera integration</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>⏳</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>BattleHUD resolves to active unit, not separately inspected unit</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>Independent inspected-unit state</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>⏳</t>
-        </is>
-      </c>
-    </row>
-    <row r="55"/>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>--- Parked Visual/Tuning ---</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>⏳</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>Right-drag sensitivity tuning</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>⏳</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>Grid readability at yaw 0 and 90 degrees</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>⏳</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>Rotated/zoomed visible-footprint camera tuning</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>⏳</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>TemplateInspector white selection outline</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>⏳</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>Startup avatar and native-control flash</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>⏳</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>Future battle-entry cinematic</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>⏳</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>Production camera-recovery buttons</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>⏳</t>
-        </is>
-      </c>
-    </row>
-    <row r="64"/>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>--- Separately Tracked Defects (not camera scope) ---</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>🐛</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>Attack confirmation regression</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>🐛</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>Tracked separately</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>BoardClient ReplicatedStorage.Modules error</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>🐛</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>Tracked separately</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>UIController initial viewport reported as 1x1</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>🐛</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>Tracked separately</t>
-        </is>
-      </c>
-    </row>
-    <row r="69"/>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>═══ SLICE 7 CROSS-SLICE BOUNDARY ═══</t>
-        </is>
-      </c>
-    </row>
-    <row r="71"/>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>Slice 7 MAY define and implement:</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Client visual composition and layout</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>SCOPE</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Battle UI phase display (consumes phase state from server, does not own transitions)</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>SCOPE</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  View Mode visual presentation (consumes inspected-unit data, does not own selection state)</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>SCOPE</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Camera presentation and input forwarding (does not own battle-input mode)</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>SCOPE</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Responsive layout</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>SCOPE</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Visual asset lookup and fallback behavior</t>
-        </is>
-      </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>SCOPE</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Display contracts for preview, timeline, status, log, unit, tile, object, and battlefield-condition data</t>
-        </is>
-      </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>SCOPE</t>
-        </is>
-      </c>
-    </row>
-    <row r="80"/>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>Slice 7 MUST NOT define or modify:</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Combat formulas</t>
-        </is>
-      </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>BOUNDARY</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Action legality</t>
-        </is>
-      </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>BOUNDARY</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Movement legality</t>
-        </is>
-      </c>
-      <c r="B84" t="inlineStr">
-        <is>
-          <t>BOUNDARY</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Target legality</t>
-        </is>
-      </c>
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>BOUNDARY</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  CT or RT calculations</t>
-        </is>
-      </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>BOUNDARY</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Status behavior</t>
-        </is>
-      </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>BOUNDARY</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Weather behavior</t>
-        </is>
-      </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>BOUNDARY</t>
-        </is>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Crisis behavior</t>
-        </is>
-      </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>BOUNDARY</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Time progression rules</t>
-        </is>
-      </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>BOUNDARY</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Event scheduling rules</t>
-        </is>
-      </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>BOUNDARY</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Summon-duration rules</t>
-        </is>
-      </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>BOUNDARY</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Object interaction rules</t>
-        </is>
-      </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>BOUNDARY</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Server-authoritative action results</t>
-        </is>
-      </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>BOUNDARY</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Database content</t>
-        </is>
-      </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>BOUNDARY</t>
-        </is>
-      </c>
-    </row>
-    <row r="96"/>
-    <row r="97">
-      <c r="A97" t="inlineStr">
-        <is>
-          <t>Fallback rule: When required presentation data is unavailable, report the missing field and render a safe fallback or omit the field. Do not calculate authoritative values on the client to complete a panel.</t>
-        </is>
-      </c>
-      <c r="B97" t="inlineStr">
-        <is>
-          <t>RULE</t>
-        </is>
-      </c>
-      <c r="C97" t="inlineStr">
-        <is>
-          <t>Locked</t>
-        </is>
-      </c>
-    </row>
-    <row r="98"/>
-    <row r="99">
-      <c r="A99" t="inlineStr">
-        <is>
-          <t>═══ SLICE OWNERSHIP ═══</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="inlineStr">
-        <is>
-          <t>Functional Scope</t>
-        </is>
-      </c>
-      <c r="B100" t="inlineStr">
-        <is>
-          <t>VISUALS, LAYOUT, THEMES, ASSETS, AND PRESENTATION ONLY. UI composition, responsive layout, theme/colors/typography, portraits/icons/models, terrain materials, prop visuals, lighting, animations, VFX, floating numbers, timeline appearance, battle log appearance, camera presentation, audio, missing-asset fallbacks</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="inlineStr">
-        <is>
-          <t>Owned Module Group</t>
-        </is>
-      </c>
-      <c r="B101" t="inlineStr">
-        <is>
-          <t>BattleHUD.lua, Theme.lua, UIConstants.lua, UIFormatting.lua, UIComponents.lua, UILayoutCoordinator.lua, UIController.client.lua, UnitInspectorPanel.client.lua, CameraController.lua (camera/presentation only)</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" t="inlineStr">
-        <is>
-          <t>Shared Integration Modules</t>
-        </is>
-      </c>
-      <c r="B102" t="inlineStr">
-        <is>
-          <t>BattleVisualClient.client.lua (read only — presentation hooks require approval)</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" t="inlineStr">
-        <is>
-          <t>Protected Dependencies</t>
-        </is>
-      </c>
-      <c r="B103" t="inlineStr">
-        <is>
-          <t>All slices (consumes their public events and APIs for display)</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" t="inlineStr">
-        <is>
-          <t>Public Contracts Provided</t>
-        </is>
-      </c>
-      <c r="B104" t="inlineStr">
-        <is>
-          <t>Visual rendering, user input intent (forwarded to server), display fallbacks</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" t="inlineStr">
-        <is>
-          <t>Public Contracts Consumed</t>
-        </is>
-      </c>
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>Battle phase state, active unit, targets, preview values, timeline, status, inventory, equipment, map state — all as read-only display data</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" t="inlineStr">
-        <is>
-          <t>Forbidden Changes</t>
-        </is>
-      </c>
-      <c r="B106" t="inlineStr">
-        <is>
-          <t>Must not modify: combat formulas, movement/target legality, CT/RT, command validation, skill/status resolution, timeline ordering, save/load, inventory/equipment transactions, recruitment/tavern/blacksmith/quest logic, map generation, content definitions, CTRBLXAI.db</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" t="inlineStr">
-        <is>
-          <t>Minimum Regression Gate</t>
-        </is>
-      </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>Minimum cross-slice smoke test + focused camera regression for camera changes</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" t="inlineStr">
-        <is>
-          <t>Checkpoint Commit</t>
-        </is>
-      </c>
-      <c r="B108" t="inlineStr">
-        <is>
-          <t>🔄 In Progress — Stage 1 Desktop Checkpoint: e8dcc977</t>
-        </is>
-      </c>
-    </row>
-    <row r="109"/>
-    <row r="110">
-      <c r="A110" t="inlineStr">
-        <is>
-          <t>═══ STAGE 2A: ROSTER AND UNIT LOADOUT PRESENTATION ═══</t>
-        </is>
-      </c>
-    </row>
-    <row r="111"/>
-    <row r="112">
-      <c r="A112" t="inlineStr">
-        <is>
-          <t>Goal:</t>
-        </is>
-      </c>
-      <c r="B112" t="inlineStr">
-        <is>
-          <t>Three-tab Loadout Hub (Info / Equipment / Skills) with persistent unit header, responsive layout, Theme-consistent presentation. Full spec in DB: loadout_ui_spec (59 rules).</t>
-        </is>
-      </c>
-    </row>
-    <row r="113"/>
-    <row r="114">
-      <c r="A114" t="inlineStr">
-        <is>
-          <t>--- Shared Navigation ---</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" t="inlineStr">
-        <is>
-          <t>Three tabs at top: INFO | EQUIPMENT | SKILLS</t>
-        </is>
-      </c>
-      <c r="B115" t="inlineStr">
-        <is>
-          <t>🔄</t>
-        </is>
-      </c>
-      <c r="C115" t="inlineStr">
-        <is>
-          <t>LoadoutScreen.lua implements tab structure</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" t="inlineStr">
-        <is>
-          <t>Persistent unit header: portrait, name, level, race, doctrine, 3x2 stat grid</t>
-        </is>
-      </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>🔄</t>
-        </is>
-      </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>LoadoutScreen.lua implements header</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" t="inlineStr">
-        <is>
-          <t>Previous/next unit controls + tap-portrait unit selector</t>
-        </is>
-      </c>
-      <c r="B117" t="inlineStr">
-        <is>
-          <t>🔄</t>
-        </is>
-      </c>
-      <c r="C117" t="inlineStr">
-        <is>
-          <t>LoadoutScreen.lua implements unit switching</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" t="inlineStr">
-        <is>
-          <t>Unit switching preserves tab, refreshes all data, clears stale selections</t>
-        </is>
-      </c>
-      <c r="B118" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" t="inlineStr">
-        <is>
-          <t>Pending-change guard on unit switch (confirm/cancel/discard)</t>
-        </is>
-      </c>
-      <c r="B119" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="120"/>
-    <row r="121">
-      <c r="A121" t="inlineStr">
-        <is>
-          <t>--- Info Tab ---</t>
-        </is>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" t="inlineStr">
-        <is>
-          <t>Primary stats with breakdown (base, allocation, equipment, doctrine)</t>
-        </is>
-      </c>
-      <c r="B122" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="C122" t="inlineStr">
-        <is>
-          <t>STR INT DEX / AGI VIT LUK</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" t="inlineStr">
-        <is>
-          <t>Stat allocation controls (only in Info)</t>
-        </is>
-      </c>
-      <c r="B123" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="C123" t="inlineStr">
-        <is>
-          <t>No respec — Slice 7 must not implement</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" t="inlineStr">
-        <is>
-          <t>Secondary stats display with authoritative breakdown on select</t>
-        </is>
-      </c>
-      <c r="B124" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="C124" t="inlineStr">
-        <is>
-          <t>No Critical Rate, Critical Damage, Evasion</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" t="inlineStr">
-        <is>
-          <t>Race info: icon, name, growth rates, Race Perk, Race Drawback</t>
-        </is>
-      </c>
-      <c r="B125" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="C125" t="inlineStr">
-        <is>
-          <t>Separate labels from Unit Perk/Drawback</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" t="inlineStr">
-        <is>
-          <t>Generated unit traits: one Perk, one Drawback</t>
-        </is>
-      </c>
-      <c r="B126" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" t="inlineStr">
-        <is>
-          <t>Doctrine summary (display-only, managed from Equipment)</t>
-        </is>
-      </c>
-      <c r="B127" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" t="inlineStr">
-        <is>
-          <t>Unit records (only when authoritative data exists)</t>
-        </is>
-      </c>
-      <c r="B128" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="129"/>
-    <row r="130">
-      <c r="A130" t="inlineStr">
-        <is>
-          <t>--- Equipment Tab ---</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" t="inlineStr">
-        <is>
-          <t>Inventory grid (left) + loadout (right) layout</t>
-        </is>
-      </c>
-      <c r="B131" t="inlineStr">
-        <is>
-          <t>🔄</t>
-        </is>
-      </c>
-      <c r="C131" t="inlineStr">
-        <is>
-          <t>LoadoutScreen.lua implements inventory grid</t>
-        </is>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" t="inlineStr">
-        <is>
-          <t>Complete loadout: MainHand, OffHand, Head, Torso, Arms, Legs, Accessory, 6 Consumable slots, Doctrine</t>
-        </is>
-      </c>
-      <c r="B132" t="inlineStr">
-        <is>
-          <t>🔄</t>
-        </is>
-      </c>
-      <c r="C132" t="inlineStr">
-        <is>
-          <t>LoadoutScreen.lua implements equipment slots</t>
-        </is>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" t="inlineStr">
-        <is>
-          <t>Off-Hand disabled when 2H equipped</t>
-        </is>
-      </c>
-      <c r="B133" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" t="inlineStr">
-        <is>
-          <t>Consumable slots 1-3 usable, 4-6 visible locked with explanation</t>
-        </is>
-      </c>
-      <c r="B134" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" t="inlineStr">
-        <is>
-          <t>Doctrine: mandatory, swap-only, cannot be empty or unequipped</t>
-        </is>
-      </c>
-      <c r="B135" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" t="inlineStr">
-        <is>
-          <t>Item-type filters, rarity filter, sorting, search</t>
-        </is>
-      </c>
-      <c r="B136" t="inlineStr">
-        <is>
-          <t>🔄</t>
-        </is>
-      </c>
-      <c r="C136" t="inlineStr">
-        <is>
-          <t>LoadoutScreen.lua implements filters</t>
-        </is>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" t="inlineStr">
-        <is>
-          <t>Item selection → comparison → equip/replace/swap transaction</t>
-        </is>
-      </c>
-      <c r="B137" t="inlineStr">
-        <is>
-          <t>🔄</t>
-        </is>
-      </c>
-      <c r="C137" t="inlineStr">
-        <is>
-          <t>LoadoutScreen.BuildItemDetail exists</t>
-        </is>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" t="inlineStr">
-        <is>
-          <t>BP never shown in any player-facing UI</t>
-        </is>
-      </c>
-      <c r="B138" t="inlineStr">
-        <is>
-          <t>RULE</t>
-        </is>
-      </c>
-      <c r="C138" t="inlineStr">
-        <is>
-          <t>Locked</t>
-        </is>
-      </c>
-    </row>
-    <row r="139"/>
-    <row r="140">
-      <c r="A140" t="inlineStr">
-        <is>
-          <t>--- Equipment Comparison ---</t>
-        </is>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" t="inlineStr">
-        <is>
-          <t>Current vs selected, only changed values</t>
-        </is>
-      </c>
-      <c r="B141" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="C141" t="inlineStr">
-        <is>
-          <t>Colors reflect gameplay consequence, not just math sign</t>
-        </is>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" t="inlineStr">
-        <is>
-          <t>Authoritative before-and-after from Slice 4 — no independent calculation</t>
-        </is>
-      </c>
-      <c r="B142" t="inlineStr">
-        <is>
-          <t>RULE</t>
-        </is>
-      </c>
-      <c r="C142" t="inlineStr">
-        <is>
-          <t>Locked</t>
-        </is>
-      </c>
-    </row>
-    <row r="143"/>
-    <row r="144">
-      <c r="A144" t="inlineStr">
-        <is>
-          <t>--- Doctrine Comparison ---</t>
-        </is>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" t="inlineStr">
-        <is>
-          <t>Swap Doctrine only (no Unequip). Warn if Doctrine Skill in Slot 1 affected</t>
-        </is>
-      </c>
-      <c r="B145" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="146"/>
-    <row r="147">
-      <c r="A147" t="inlineStr">
-        <is>
-          <t>--- Skills Tab ---</t>
-        </is>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" t="inlineStr">
-        <is>
-          <t>Five Skill rows: slot, icon, name, effect, MP, RT, 2 augment slots each</t>
-        </is>
-      </c>
-      <c r="B148" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" t="inlineStr">
-        <is>
-          <t>Slot 1: Doctrine Skill (3 choices from doctrine, player selects one)</t>
-        </is>
-      </c>
-      <c r="B149" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="C149" t="inlineStr">
-        <is>
-          <t>Cannot accept normal Skill Card</t>
-        </is>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" t="inlineStr">
-        <is>
-          <t>Slots 2-4: Skill Cards with 2 Augment slots each</t>
-        </is>
-      </c>
-      <c r="B150" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" t="inlineStr">
-        <is>
-          <t>Slot 5: visible locked — 'Locked by First Race Evolution'</t>
-        </is>
-      </c>
-      <c r="B151" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" t="inlineStr">
-        <is>
-          <t>Skill Card + Augment Card inventory with subtabs, stacking</t>
-        </is>
-      </c>
-      <c r="B152" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" t="inlineStr">
-        <is>
-          <t>Skill Card details: full authoritative fields, formulas displayed not evaluated</t>
-        </is>
-      </c>
-      <c r="B153" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" t="inlineStr">
-        <is>
-          <t>Augment Card details: compatibility from functional system, modified costs shown</t>
-        </is>
-      </c>
-      <c r="B154" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" t="inlineStr">
-        <is>
-          <t>Filters: type, tags, element, compatibility</t>
-        </is>
-      </c>
-      <c r="B155" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="156"/>
-    <row r="157">
-      <c r="A157" t="inlineStr">
-        <is>
-          <t>--- Interaction ---</t>
-        </is>
-      </c>
-    </row>
-    <row r="158">
-      <c r="A158" t="inlineStr">
-        <is>
-          <t>Desktop: drag-and-drop + click-to-select for Skills/Augments</t>
-        </is>
-      </c>
-      <c r="B158" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" t="inlineStr">
-        <is>
-          <t>Mobile: tap → highlight destinations → tap destination → preview → confirm</t>
-        </is>
-      </c>
-      <c r="B159" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="C159" t="inlineStr">
-        <is>
-          <t>Drag must not be only method</t>
-        </is>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" t="inlineStr">
-        <is>
-          <t>Pending change preview before all commits</t>
-        </is>
-      </c>
-      <c r="B160" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="161"/>
-    <row r="162">
-      <c r="A162" t="inlineStr">
-        <is>
-          <t>--- Responsive ---</t>
-        </is>
-      </c>
-    </row>
-    <row r="163">
-      <c r="A163" t="inlineStr">
-        <is>
-          <t>Mobile-first layout, desktop expanded</t>
-        </is>
-      </c>
-      <c r="B163" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="164">
-      <c r="A164" t="inlineStr">
-        <is>
-          <t>Roblox controls unobstructed, tabs at top, no full rebuild on switch</t>
-        </is>
-      </c>
-      <c r="B164" t="inlineStr">
-        <is>
-          <t>RULE</t>
-        </is>
-      </c>
-      <c r="C164" t="inlineStr">
-        <is>
-          <t>Locked</t>
-        </is>
-      </c>
-    </row>
-    <row r="165"/>
-    <row r="166">
-      <c r="A166" t="inlineStr">
-        <is>
-          <t>--- Loadout Presentation Completion Gate ---</t>
-        </is>
-      </c>
-    </row>
-    <row r="167">
-      <c r="A167" t="inlineStr">
-        <is>
-          <t>Three tabs consistent, Roblox controls clear, unit switching works</t>
-        </is>
-      </c>
-      <c r="B167" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="168">
-      <c r="A168" t="inlineStr">
-        <is>
-          <t>Info: accurate stats, allocation only in Info, no nonexistent stats</t>
-        </is>
-      </c>
-      <c r="B168" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="169">
-      <c r="A169" t="inlineStr">
-        <is>
-          <t>Equipment: square cards, no BP, accurate comparison, doctrine swap-only</t>
-        </is>
-      </c>
-      <c r="B169" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="170">
-      <c r="A170" t="inlineStr">
-        <is>
-          <t>Skills: doctrine skill slot 1, skill cards 2-4, locked slot 5, augment slots</t>
-        </is>
-      </c>
-      <c r="B170" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="171">
-      <c r="A171" t="inlineStr">
-        <is>
-          <t>Mobile tap-based management works, desktop drag works</t>
-        </is>
-      </c>
-      <c r="B171" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="172">
-      <c r="A172" t="inlineStr">
-        <is>
-          <t>Pending changes cannot be silently lost</t>
-        </is>
-      </c>
-      <c r="B172" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="173">
-      <c r="A173" t="inlineStr">
-        <is>
-          <t>No Slice 7 interface calculates authoritative gameplay values</t>
-        </is>
-      </c>
-      <c r="B173" t="inlineStr">
-        <is>
-          <t>RULE</t>
-        </is>
-      </c>
-    </row>
-    <row r="174">
-      <c r="A174" t="inlineStr">
-        <is>
-          <t>Save and reload preserve all committed loadout changes</t>
-        </is>
-      </c>
-      <c r="B174" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" t="inlineStr">
-        <is>
-          <t>═══ STAGE 2B: BATTLE HUD EXPANSION (tracked post-audit) ═══</t>
-        </is>
-      </c>
-      <c r="B176" t="inlineStr"/>
-      <c r="C176" t="inlineStr"/>
-    </row>
-    <row r="177">
-      <c r="A177" t="inlineStr"/>
-      <c r="B177" t="inlineStr"/>
-      <c r="C177" t="inlineStr"/>
-    </row>
-    <row r="178">
-      <c r="A178" t="inlineStr">
-        <is>
-          <t>BattleHUD.lua expanded to 66KB (from 37KB baseline)</t>
-        </is>
-      </c>
-      <c r="B178" t="inlineStr">
-        <is>
-          <t>🔄</t>
-        </is>
-      </c>
-      <c r="C178" t="inlineStr">
-        <is>
-          <t>Major expansion: actor/target cards, skill list, damage preview, tile info, battle log, phase display, tooltips, confirm bar</t>
-        </is>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" t="inlineStr">
-        <is>
-          <t>Theme.lua expanded to 20KB (from 7KB baseline)</t>
-        </is>
-      </c>
-      <c r="B179" t="inlineStr">
-        <is>
-          <t>🔄</t>
-        </is>
-      </c>
-      <c r="C179" t="inlineStr">
-        <is>
-          <t>Expanded color palette, rarity colors, spacing tokens</t>
-        </is>
-      </c>
-    </row>
-    <row r="180">
-      <c r="A180" t="inlineStr">
-        <is>
-          <t>BattleVisualClient.lua expanded to 83KB (from 62KB baseline)</t>
-        </is>
-      </c>
-      <c r="B180" t="inlineStr">
-        <is>
-          <t>🔄</t>
-        </is>
-      </c>
-      <c r="C180" t="inlineStr">
-        <is>
-          <t>LoadoutScreen integration, expanded event handlers</t>
-        </is>
-      </c>
-    </row>
-    <row r="181">
-      <c r="A181" t="inlineStr">
-        <is>
-          <t>UnitInspectorPanel.lua at 24KB</t>
-        </is>
-      </c>
-      <c r="B181" t="inlineStr">
-        <is>
-          <t>🔄</t>
-        </is>
-      </c>
-      <c r="C181" t="inlineStr">
-        <is>
-          <t>3-tab inspector (Stats/Equipment/Skills)</t>
-        </is>
-      </c>
-    </row>
-    <row r="182">
-      <c r="A182" t="inlineStr"/>
-      <c r="B182" t="inlineStr"/>
-      <c r="C182" t="inlineStr"/>
-    </row>
-    <row r="183">
-      <c r="A183" t="inlineStr">
-        <is>
-          <t>--- New Modules Created ---</t>
-        </is>
-      </c>
-      <c r="B183" t="inlineStr"/>
-      <c r="C183" t="inlineStr"/>
-    </row>
-    <row r="184">
-      <c r="A184" t="inlineStr">
-        <is>
-          <t>LoadoutScreen.lua (76KB) — full loadout UI implementation</t>
-        </is>
-      </c>
-      <c r="B184" t="inlineStr">
-        <is>
-          <t>🔄</t>
-        </is>
-      </c>
-      <c r="C184" t="inlineStr">
-        <is>
-          <t>Slice 7 Stage 2A</t>
-        </is>
-      </c>
-    </row>
-    <row r="185">
-      <c r="A185" t="inlineStr">
-        <is>
-          <t>MockLoadoutData.lua (25KB) — test data for loadout development</t>
-        </is>
-      </c>
-      <c r="B185" t="inlineStr">
-        <is>
-          <t>🔄</t>
-        </is>
-      </c>
-      <c r="C185" t="inlineStr">
-        <is>
-          <t>Development aid</t>
-        </is>
-      </c>
-    </row>
-    <row r="186">
-      <c r="A186" t="inlineStr">
-        <is>
-          <t>LoadoutController.client.lua (2KB) — entry point, L key toggle</t>
-        </is>
-      </c>
-      <c r="B186" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="C186" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C80"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Goal:</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>After returning from battle, the player can use the Guild Base to recruit and manage units, access services, improve facilities, select activities, purchase or earn progression items, and prepare for future battles.</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Done When:</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Guild Base hub is functional: recruitment, merchants, services, quests, dispatch, explore all operational with authoritative rules. All acquisitions persist through Slice 4 APIs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Task</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Guild Base navigation and functional hub state</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Recruitment transactions</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Tavern services</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Guild progression (Guild XP, Guild Level)</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Locked direction in DB: loot_progression / Guild Progression</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Facility upgrades</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Blacksmith services</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Locked direction: facility level, recipes, materials, no LUK</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Out-of-battle merchants</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Locked direction: Guild/service progression, region, unlocks, no LUK</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Skill management beyond basic persistent loadout storage</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Doctrine management and acquisition</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Skill Card management and acquisition</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Augment Card management and acquisition</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Quest board</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Quest types locked: bring-me, battle, arena, boss, protect, survive, defeat X</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Dispatch</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Locked: predetermined rewards shown before acceptance</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Explore</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Service costs and transactions</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Merchant prices and transactions</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Unlocks and prerequisites</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Transition from Guild Base to battle preparation</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>═══ ACQUIRABLE CONTENT ═══</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Equipment — battle loot, quest rewards, activity rewards, merchant purchases</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Rules from Game Rules; definitions from Slice 6</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Consumables — battle loot, quest rewards, activity rewards, merchant purchases</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>140 items defined in consumable_items</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Doctrines — quest rewards, activity rewards, merchant purchases</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Duplicates valid per locked rule</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Skill Cards — quest rewards, activity rewards, merchant purchases</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Augment Cards — quest rewards, activity rewards, merchant purchases</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Acquisition eligibility, rarity, probabilities, prices per authoritative Game Rules</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>RULE</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Do not invent missing values</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>═══ ACQUISITION SOURCE BOUNDARY ═══</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Battle loot: generated and committed through Slice 4 reward + inventory transaction</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>RULE</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Slice 4 owned. Reward pipeline in reward_generation (10-step).</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Quest/Dispatch/Explore/activity rewards: determined by Slice 8, handed to Slice 4 APIs</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>RULE</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Slice 8 validates → Slice 4 persists</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Merchant purchases: availability/price/validation = Slice 8; persistence = Slice 4</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>RULE</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Town services use Guild Level, not LUK (locked)</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Content definitions: consumed from Slice 6 + Game Rules — Slice 8 does not redefine</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>RULE</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>═══ PERSISTENCE RULE ═══</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>Slice 8 must NOT maintain a second inventory, roster, equipment, Skill, Doctrine, or Augment ownership database</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>RULE</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>Acquisition flow: Slice 8 validates → Slice 8 produces result → Slice 4 records ownership → Slice 4 saves → Slice 7 presents</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>RULE</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>Unsuccessful transaction must not create or persist ownership</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>RULE</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>═══ EXISTING AUTHORITATIVE RULES IN DB ═══</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>Loot Rarity Weights: Normal and Elite encounter tables (locked)</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>EXISTS</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>loot_progression table</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>Reward Sequence: 6-step pipeline with rarity ceilings per source (locked)</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>EXISTS</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>loot_progression table</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>Activities and Loot: drop chances, Fortune rules, categories, Doctrine/Skill/Augment reward directions (locked)</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>EXISTS</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>loot_progression table</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>Guild Progression: Guild XP, Guild Level gates merchants/recruitment/blacksmith/facilities (locked direction)</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>EXISTS</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>loot_progression table</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>Elite Loot Rules: separate encounter and reward rules (locked)</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>EXISTS</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>loot_progression table</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>Gold Fortune: applies-to and doesn't-apply-to lists (locked)</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>EXISTS</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>loot_progression table</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>Service Boundaries: Reward Service and other service scopes defined</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>EXISTS</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>service_boundaries table</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>Consumable Framework + 140 items with full schemas</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>EXISTS</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>consumable_framework + consumable_items tables</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>Reward Generation Pipeline: 10-step opportunity-to-commit pipeline</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>EXISTS</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>reward_generation table</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>═══ SPECIFIC VALUES NOT YET AUTHORED ═══</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>Merchant inventories (which items, quantities)</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>UNDEFINED</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>Direction locked; specifics pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>Merchant prices</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>UNDEFINED</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>Merchant refresh rates and behavior</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>UNDEFINED</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>Recruitment pools and generation rules</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>UNDEFINED</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>Direction locked; specifics pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>Facility upgrade costs and tier progression</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>UNDEFINED</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>Blacksmith recipes and material requirements</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>UNDEFINED</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>Direction locked; specifics pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>Quest reward tables (specific rewards per quest)</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>UNDEFINED</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>Dispatch reward pools</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>UNDEFINED</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>Predetermined rewards shown before acceptance (locked)</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>Explore reward pools</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>UNDEFINED</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>Guild XP amounts per activity</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>UNDEFINED</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>Low-level farming sharply reduced (locked direction); exact bands pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>Elite encounter appearance rate</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>UNDEFINED</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>Locked as rare random; exact rate pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>═══ SLICE OWNERSHIP ═══</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>Functional Scope</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>Guild Base framework, merchants, purchases, recruitment, quest/activity rewards, Doctrine/Skill Card/Augment Card acquisition workflows, Tavern, Blacksmith, facility, Guild progression, management workflows, service costs, unlocks, battle-prep transition</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>Slice 4 Dependencies</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>Inventory ownership, roster ownership, equipment/loadout state, equip/unequip, save/load, adding acquired items to persistent inventory, restoring after rejoin, battle reward commitment, minimal functional Loadout Hub</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>Slice 6 Dependencies</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>Content catalogs: equipment, consumables, Doctrines, Skill Cards, Augment Cards</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>Slice 7 Dependencies</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>Guild Base visual presentation, merchant-screen layout, reward/acquisition presentation, item/Doctrine/Skill Card/Augment Card visual components, icons, portraits, rarity, themes, animations, VFX, responsive layout, UI sound</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>Forbidden Changes</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>Must not duplicate Slice 4 persistence, redefine Slice 6 content, or build Slice 7 presentation</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>═══ BLOCKERS AND STATUS ═══</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>Locked frameworks and directions exist in DB — Slice 8 is not starting from zero</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>INFO</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>loot_progression, reward_generation, consumable_framework, service_boundaries</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>Specific service values (prices, inventories, refresh, recipes, pools, costs) are not yet authored</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>PARTIAL</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>Design work needed for numerical values; locked directions provide the constraints</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>Slice 4 persistence APIs must be functional before Slice 8 can commit acquisitions</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>DEP</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t>Slice 6 content catalogs must exist before merchants can offer items</t>
-        </is>
-      </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>DEP</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>Checkpoint Commit</t>
-        </is>
-      </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>⬜ Not Started</t>
         </is>
       </c>
     </row>
@@ -5772,7 +3536,6 @@
         </is>
       </c>
     </row>
-    <row r="36"/>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
@@ -5797,7 +3560,6 @@
         </is>
       </c>
     </row>
-    <row r="39"/>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
@@ -5890,7 +3652,6 @@
         </is>
       </c>
     </row>
-    <row r="46"/>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
@@ -5961,7 +3722,6 @@
         </is>
       </c>
     </row>
-    <row r="52"/>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
@@ -6015,7 +3775,6 @@
         </is>
       </c>
     </row>
-    <row r="57"/>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
@@ -6115,7 +3874,6 @@
         </is>
       </c>
     </row>
-    <row r="65"/>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
@@ -6412,7 +4170,6 @@
         </is>
       </c>
     </row>
-    <row r="84"/>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>

</xml_diff>